<commit_message>
Add remaining judgements with question style switching
</commit_message>
<xml_diff>
--- a/debug/judgements_q_sty_swi/excel_overviews/gpt-4.1_vs_Llama-2-7b-chat-hf/Qwen3-4B-Instruct-2507/aae/total_votes_file.xlsx
+++ b/debug/judgements_q_sty_swi/excel_overviews/gpt-4.1_vs_Llama-2-7b-chat-hf/Qwen3-4B-Instruct-2507/aae/total_votes_file.xlsx
@@ -430,13 +430,13 @@
         <v>7</v>
       </c>
       <c r="C2">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D2">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G2">
         <v>8</v>
@@ -450,16 +450,16 @@
         <v>8</v>
       </c>
       <c r="C3">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D3">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="G3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H3">
         <v>852</v>

</xml_diff>